<commit_message>
chore(bh): AccID 欄加寬並在標題加註「MGID 填 API ID」
範本的 B 欄標題改為「AccID（MGID 填 API ID）」，欄寬 10.8 → 30
（放得下標題註解與最長的範例值 CPM_MundoPixarExperience）。

⚠️ 標題文字就是程式取欄位的鍵（row.get('AccID')），直接改會噴
Missing required columns: AccID；而且 AE 手上還留著標題為純 'AccID' 的舊範本。
⇒ bh_service 讀檔後先用 _strip_header_note 去掉標題的括號註解（全形半形都吃），
新舊範本都收得下。

新增 tests/test_bh_service_headers.py（4 個，修改前確認為紅）。

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01MJtFR2kneiYN5FBdQpP4Mg
</commit_message>
<xml_diff>
--- a/static/bh_import_template.xlsx
+++ b/static/bh_import_template.xlsx
@@ -463,7 +463,7 @@
   <sheetFormatPr baseColWidth="10" defaultColWidth="9" defaultRowHeight="14.25" customHeight="1"/>
   <cols>
     <col width="7.19921875" bestFit="1" customWidth="1" style="2" min="1" max="1"/>
-    <col width="10.796875" customWidth="1" style="2" min="2" max="2"/>
+    <col width="30" customWidth="1" style="2" min="2" max="2"/>
     <col width="20.19921875" bestFit="1" customWidth="1" style="2" min="3" max="3"/>
     <col width="10.59765625" bestFit="1" customWidth="1" style="2" min="4" max="4"/>
     <col width="15.3984375" bestFit="1" customWidth="1" style="2" min="5" max="6"/>
@@ -481,7 +481,7 @@
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>AccID</t>
+          <t>AccID（MGID 填 API ID）</t>
         </is>
       </c>
       <c r="C1" s="1" t="inlineStr">

</xml_diff>